<commit_message>
bug n detials- landing mpage
</commit_message>
<xml_diff>
--- a/static/downloads/modelo_facturacion.xlsx
+++ b/static/downloads/modelo_facturacion.xlsx
@@ -1,55 +1,85 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Bias\ZyM_Accounting\ZyM_Accounting\static\downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11430"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facturación" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Facturación" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>FECHA EMISION</t>
+  </si>
+  <si>
+    <t>CUIT CLIENTE</t>
+  </si>
+  <si>
+    <t>RAZON SOCIAL CLIENTE</t>
+  </si>
+  <si>
+    <t>DOMICILIO CLIENTE</t>
+  </si>
+  <si>
+    <t>NOMBRE CONTACTO</t>
+  </si>
+  <si>
+    <t>DESCRIPCION / CONCEPTO</t>
+  </si>
+  <si>
+    <t>IMPORTE</t>
+  </si>
+  <si>
+    <t>COMP NRO</t>
+  </si>
+  <si>
+    <t>CAE</t>
+  </si>
+  <si>
+    <t>VENCIMIENTO</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <b/>
       <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="00C9D1D9"/>
-      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F6FEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00161B22"/>
+        <fgColor rgb="FF1F6FEB"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,103 +93,42 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="0030363D"/>
+        <color rgb="FF30363D"/>
       </left>
       <right style="thin">
-        <color rgb="0030363D"/>
+        <color rgb="FF30363D"/>
       </right>
       <top style="thin">
-        <color rgb="0030363D"/>
+        <color rgb="FF30363D"/>
       </top>
       <bottom style="thin">
-        <color rgb="0030363D"/>
+        <color rgb="FF30363D"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -447,122 +416,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FECHA EMISION</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>CUIT CLIENTE</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>RAZON SOCIAL CLIENTE</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>DOMICILIO CLIENTE</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>NOMBRE CONTACTO</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>DESCRIPCION / CONCEPTO</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>IMPORTE</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>COMP NRO</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>CAE</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>VENCIMIENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>16/02/2026</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>30-71768115-7</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Consorcio de Propietarios Malabia 1260</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Malabia 1260 - Capital Federal</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>ROMINA FRAIESE</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Descripción del trabajo realizado según presupuesto.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>404315</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>C00002-00000144</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>18/02/2026 VENCIMIENTO</t>
-        </is>
+    <row r="1" spans="1:10" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>